<commit_message>
Updated week 3 stats with player insights feature
</commit_message>
<xml_diff>
--- a/game-stats/Week1_G-MOB_vs_All-Madden.xlsx
+++ b/game-stats/Week1_G-MOB_vs_All-Madden.xlsx
@@ -1533,13 +1533,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:T23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="17" min="1" max="1"/>
     <col width="22" customWidth="1" style="17" min="2" max="2"/>
     <col width="14" customWidth="1" style="17" min="3" max="3"/>
     <col width="11" customWidth="1" style="17" min="4" max="18"/>
+    <col width="10" customWidth="1" style="17" min="11" max="11"/>
     <col width="10" customWidth="1" style="17" min="16" max="16"/>
     <col width="8.710000000000001" customWidth="1" style="17" min="19" max="27"/>
   </cols>
@@ -1595,47 +1596,52 @@
           <t>Rush YDs</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>Rush TD</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>Rush TDs</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Rec YDs</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>TDs</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Def INTs</t>
         </is>
       </c>
-      <c r="P1" s="18" t="inlineStr">
+      <c r="Q1" s="18" t="inlineStr">
         <is>
           <t>Def TDs</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>PBU</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="S1" s="9" t="inlineStr">
         <is>
           <t>Sacks</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="T1" s="9" t="inlineStr">
         <is>
           <t>Flag Pulls</t>
         </is>
@@ -1676,29 +1682,32 @@
       <c r="J2" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="14" t="n"/>
-      <c r="L2" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="14" t="n"/>
       <c r="M2" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="14" t="n">
+      <c r="N2" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="S2" s="14" t="n">
+      <c r="T2" s="14" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1737,29 +1746,32 @@
       <c r="J3" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="14" t="n"/>
-      <c r="L3" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="14" t="n"/>
       <c r="M3" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="14" t="n">
+      <c r="N3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R3" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1798,29 +1810,32 @@
       <c r="J4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="14" t="n"/>
-      <c r="L4" s="14" t="n">
+      <c r="K4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14" t="n"/>
+      <c r="M4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="N4" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="14" t="n">
+      <c r="O4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1859,29 +1874,32 @@
       <c r="J5" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="14" t="n"/>
-      <c r="L5" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="14" t="n"/>
       <c r="M5" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="14" t="n">
+      <c r="N5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R5" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1920,29 +1938,32 @@
       <c r="J6" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="K6" s="14" t="n"/>
-      <c r="L6" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="14" t="n"/>
       <c r="M6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="14" t="n">
+      <c r="N6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1981,29 +2002,32 @@
       <c r="J7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="K7" s="14" t="n"/>
-      <c r="L7" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="14" t="n"/>
       <c r="M7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="14" t="n">
+      <c r="N7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2042,29 +2066,32 @@
       <c r="J8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="14" t="n"/>
-      <c r="L8" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="14" t="n"/>
       <c r="M8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="14" t="n">
+      <c r="N8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2103,29 +2130,32 @@
       <c r="J9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="14" t="n"/>
-      <c r="L9" s="14" t="n">
+      <c r="K9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="14" t="n"/>
+      <c r="M9" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="N9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="14" t="n">
+      <c r="O9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R9" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2164,29 +2194,32 @@
       <c r="J10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="14" t="n"/>
       <c r="M10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="14" t="n">
+      <c r="N10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2225,29 +2258,32 @@
       <c r="J11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="14" t="n">
+      <c r="K11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="14" t="n"/>
+      <c r="M11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="N11" s="16" t="n">
+      <c r="O11" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="O11" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="14" t="n">
+      <c r="P11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R11" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2286,29 +2322,32 @@
       <c r="J12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="14" t="n"/>
-      <c r="L12" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="14" t="n"/>
       <c r="M12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="14" t="n">
+      <c r="N12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2347,29 +2386,32 @@
       <c r="J13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="14" t="n"/>
       <c r="M13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="14" t="n">
+      <c r="N13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R13" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2408,29 +2450,32 @@
       <c r="J14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="14" t="n"/>
       <c r="M14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="14" t="n">
+      <c r="N14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2469,29 +2514,32 @@
       <c r="J15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="14" t="n"/>
-      <c r="L15" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="14" t="n"/>
       <c r="M15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="14" t="n">
+      <c r="N15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2530,29 +2578,32 @@
       <c r="J16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="14" t="n"/>
-      <c r="L16" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="14" t="n"/>
       <c r="M16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="14" t="n">
+      <c r="N16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2591,29 +2642,32 @@
       <c r="J17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="14" t="n"/>
-      <c r="L17" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="14" t="n"/>
       <c r="M17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="14" t="n">
+      <c r="N17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2652,29 +2706,32 @@
       <c r="J18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="14" t="n"/>
-      <c r="L18" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="14" t="n"/>
       <c r="M18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="14" t="n">
+      <c r="N18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2713,29 +2770,32 @@
       <c r="J19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="14" t="n"/>
       <c r="M19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="14" t="n">
+      <c r="N19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2774,29 +2834,32 @@
       <c r="J20" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="14" t="n"/>
-      <c r="L20" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="14" t="n"/>
       <c r="M20" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="14" t="n">
+      <c r="N20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2835,29 +2898,32 @@
       <c r="J21" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="14" t="n"/>
-      <c r="L21" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="14" t="n"/>
       <c r="M21" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="14" t="n">
+      <c r="N21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R21" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2896,29 +2962,32 @@
       <c r="J22" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="14" t="n"/>
-      <c r="L22" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="14" t="n"/>
       <c r="M22" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N22" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="14" t="n">
+      <c r="N22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2957,29 +3026,32 @@
       <c r="J23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="14" t="n"/>
-      <c r="L23" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="14" t="n"/>
       <c r="M23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="14" t="n">
+      <c r="N23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R23" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3972,13 +4044,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="17" min="1" max="1"/>
     <col width="22" customWidth="1" style="17" min="2" max="2"/>
     <col width="14" customWidth="1" style="17" min="3" max="3"/>
     <col width="11" customWidth="1" style="17" min="4" max="18"/>
+    <col width="10" customWidth="1" style="17" min="11" max="11"/>
     <col width="10" customWidth="1" style="17" min="16" max="16"/>
     <col width="8.710000000000001" customWidth="1" style="17" min="19" max="27"/>
   </cols>
@@ -4034,47 +4107,52 @@
           <t>Rush YDs</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>Rush TD</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>Rush TDs</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Rec YDs</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>TDs</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Def INTs</t>
         </is>
       </c>
-      <c r="P1" s="18" t="inlineStr">
+      <c r="Q1" s="18" t="inlineStr">
         <is>
           <t>Def TDs</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="R1" s="9" t="inlineStr">
         <is>
           <t>PBU</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="S1" s="9" t="inlineStr">
         <is>
           <t>Sacks</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="T1" s="9" t="inlineStr">
         <is>
           <t>Flag Pulls</t>
         </is>
@@ -4115,29 +4193,32 @@
       <c r="J2" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K2" s="14" t="n"/>
-      <c r="L2" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="14" t="n"/>
       <c r="M2" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="14" t="n">
+      <c r="N2" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R2" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S2" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4176,29 +4257,32 @@
       <c r="J3" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="14" t="n"/>
-      <c r="L3" s="14" t="n">
+      <c r="K3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="14" t="n"/>
+      <c r="M3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="N3" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="14" t="n">
+      <c r="O3" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R3" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4237,29 +4321,32 @@
       <c r="J4" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="K4" s="14" t="n"/>
-      <c r="L4" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14" t="n"/>
       <c r="M4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="14" t="n">
+      <c r="N4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4298,29 +4385,32 @@
       <c r="J5" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="14" t="n"/>
-      <c r="L5" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="14" t="n"/>
       <c r="M5" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="14" t="n">
+      <c r="N5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R5" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4359,29 +4449,32 @@
       <c r="J6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="14" t="n"/>
-      <c r="L6" s="14" t="n">
+      <c r="K6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="14" t="n"/>
+      <c r="M6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="N6" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="14" t="n">
+      <c r="O6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4420,29 +4513,32 @@
       <c r="J7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="14" t="n"/>
-      <c r="L7" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="14" t="n"/>
       <c r="M7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="14" t="n">
+      <c r="N7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4481,29 +4577,32 @@
       <c r="J8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="14" t="n"/>
-      <c r="L8" s="14" t="n">
+      <c r="K8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="14" t="n"/>
+      <c r="M8" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M8" s="14" t="n">
+      <c r="N8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="N8" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="14" t="n">
+      <c r="O8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="S8" s="14" t="n">
+      <c r="T8" s="14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4542,29 +4641,32 @@
       <c r="J9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="14" t="n"/>
-      <c r="L9" s="14" t="n">
+      <c r="K9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="14" t="n"/>
+      <c r="M9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="N9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="14" t="n">
+      <c r="O9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="R9" s="14" t="n">
-        <v>0</v>
-      </c>
       <c r="S9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4603,29 +4705,32 @@
       <c r="J10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="14" t="n"/>
       <c r="M10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="14" t="n">
+      <c r="N10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4664,29 +4769,32 @@
       <c r="J11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="14" t="n"/>
       <c r="M11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="14" t="n">
+      <c r="N11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="S11" s="14" t="n">
+      <c r="T11" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4725,29 +4833,32 @@
       <c r="J12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="14" t="n"/>
-      <c r="L12" s="14" t="n">
+      <c r="K12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="14" t="n"/>
+      <c r="M12" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="N12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="14" t="n">
+      <c r="O12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4786,29 +4897,32 @@
       <c r="J13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="14" t="n"/>
       <c r="M13" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="14" t="n">
+      <c r="N13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R13" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4847,29 +4961,32 @@
       <c r="J14" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="14" t="n">
+      <c r="K14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="14" t="n"/>
+      <c r="M14" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="M14" s="14" t="n">
+      <c r="N14" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="N14" s="16" t="n">
+      <c r="O14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="O14" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="14" t="n">
+      <c r="P14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4908,29 +5025,32 @@
       <c r="J15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="14" t="n"/>
-      <c r="L15" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="14" t="n"/>
       <c r="M15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="14" t="n">
+      <c r="N15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4969,29 +5089,32 @@
       <c r="J16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="14" t="n"/>
-      <c r="L16" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="14" t="n"/>
       <c r="M16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="14" t="n">
+      <c r="N16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5030,29 +5153,32 @@
       <c r="J17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="14" t="n"/>
-      <c r="L17" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="14" t="n"/>
       <c r="M17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="14" t="n">
+      <c r="N17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5091,29 +5217,32 @@
       <c r="J18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="14" t="n"/>
-      <c r="L18" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="14" t="n"/>
       <c r="M18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="14" t="n">
+      <c r="N18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5152,29 +5281,32 @@
       <c r="J19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="14" t="n">
+      <c r="K19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="14" t="n"/>
+      <c r="M19" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M19" s="14" t="n">
+      <c r="N19" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="N19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="14" t="n">
+      <c r="O19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5213,29 +5345,32 @@
       <c r="J20" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="14" t="n"/>
-      <c r="L20" s="14" t="n">
-        <v>0</v>
-      </c>
+      <c r="K20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="14" t="n"/>
       <c r="M20" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="14" t="n">
+      <c r="N20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="19" t="n">
         <v>0</v>
       </c>
       <c r="R20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="S20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>